<commit_message>
changed to adum parts in trenz library
</commit_message>
<xml_diff>
--- a/manufacturing reports/BOM/bom_change_s001.xlsx
+++ b/manufacturing reports/BOM/bom_change_s001.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t>ISO7741QDWRQ1</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>ADUM4402BRWZ</t>
-  </si>
-  <si>
-    <t>yes</t>
   </si>
   <si>
     <t>no</t>
@@ -446,7 +443,7 @@
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -460,7 +457,7 @@
         <v>15</v>
       </c>
       <c r="D2">
-        <v>31501</v>
+        <v>31526</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>13</v>
@@ -480,13 +477,13 @@
         <v>16</v>
       </c>
       <c r="D3">
-        <v>31502</v>
+        <v>31527</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -504,7 +501,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -522,7 +519,7 @@
         <v>12</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -540,7 +537,7 @@
         <v>9</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>